<commit_message>
feat: expand intelligence APIs, ingestion pipelines, and web console
</commit_message>
<xml_diff>
--- a/investai.xlsx
+++ b/investai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\invest_ai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5A1F03-7496-493B-90EB-5CBC7C06E37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D999B8F9-9616-46D0-AB78-10B562F64120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12600" windowHeight="15150" activeTab="2" xr2:uid="{F5D4FDE9-00C8-4EAA-8556-5AECFB8EB8A2}"/>
+    <workbookView xWindow="12600" yWindow="0" windowWidth="12600" windowHeight="15150" activeTab="1" xr2:uid="{F5D4FDE9-00C8-4EAA-8556-5AECFB8EB8A2}"/>
   </bookViews>
   <sheets>
     <sheet name="개요" sheetId="1" r:id="rId1"/>
@@ -577,438 +577,439 @@
     <t>미국 CPI/PPI/고용 등 시계열 API</t>
   </si>
   <si>
+    <t>Batch + Event</t>
+  </si>
+  <si>
+    <t>일 1회 + 발표일 전후 집중</t>
+  </si>
+  <si>
+    <t>CPI/PPI 등 시계열(Series 기반)</t>
+  </si>
+  <si>
+    <t>원천기관 API. 발표값/일정은 별도 릴리즈 페이지/스케줄과 결합 권장.</t>
+  </si>
+  <si>
+    <t>https://www.bls.gov/developers/</t>
+  </si>
+  <si>
+    <t>미국 CPI 릴리즈 페이지/문서</t>
+  </si>
+  <si>
+    <t>BLS CPI News Release</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>발표 전후 30초~2분 폴링</t>
+  </si>
+  <si>
+    <t>릴리즈 본문/표/첨부</t>
+  </si>
+  <si>
+    <t>정책/문구 변화 요약에 LLM 사용 가능. 일정 변경 공지 확인 필요.</t>
+  </si>
+  <si>
+    <t>https://www.bls.gov/news.release/cpi.htm</t>
+  </si>
+  <si>
+    <t>미국 GDP/PCE 등</t>
+  </si>
+  <si>
+    <t>BEA API / Release Schedule</t>
+  </si>
+  <si>
+    <t>OpenAPI + Web/JSON/ICS</t>
+  </si>
+  <si>
+    <t>일 1회 + 발표 전후 집중</t>
+  </si>
+  <si>
+    <t>GDP, PCE 등 지표값 및 릴리즈 일정</t>
+  </si>
+  <si>
+    <t>스케줄 JSON/ICS 활용 가능. 개정치(revisions) 처리 고려.</t>
+  </si>
+  <si>
+    <t>https://www.bea.gov/resources/for-developers</t>
+  </si>
+  <si>
+    <t>경제 데이터 통합 허브(백테스트/리비전)</t>
+  </si>
+  <si>
+    <t>FRED API (ALFRED 포함)</t>
+  </si>
+  <si>
+    <t>Federal Reserve (Official)</t>
+  </si>
+  <si>
+    <t>다양한 경제지표 시계열, vintage(리비전) 데이터(옵션)</t>
+  </si>
+  <si>
+    <t>원천기관 대비 중계 레이어. 실시간 발표 해석은 원천기관 우선 권장.</t>
+  </si>
+  <si>
+    <t>https://fred.stlouisfed.org/docs/api/fred/</t>
+  </si>
+  <si>
+    <t>공시</t>
+  </si>
+  <si>
+    <t>한국 공시 원천/원문/XML</t>
+  </si>
+  <si>
+    <t>OPENDART (금감원)</t>
+  </si>
+  <si>
+    <t>Regulator (Official)</t>
+  </si>
+  <si>
+    <t>Polling + On-demand</t>
+  </si>
+  <si>
+    <t>장중/장후 1~3분 폴링 + 원문 즉시 다운로드</t>
+  </si>
+  <si>
+    <t>공시목록, 공시원문(XML/첨부), 정정공시</t>
+  </si>
+  <si>
+    <t>corp_code 매핑 필요. 정정공시 체인 관리 필수.</t>
+  </si>
+  <si>
+    <t>https://opendart.fss.or.kr/</t>
+  </si>
+  <si>
+    <t>거래소 고유공시/투자유의/IR 보완</t>
+  </si>
+  <si>
+    <t>Primary(보완)</t>
+  </si>
+  <si>
+    <t>KRX KIND</t>
+  </si>
+  <si>
+    <t>Web (파싱)</t>
+  </si>
+  <si>
+    <t>2~5분(공시), 1~3분(투자유의)</t>
+  </si>
+  <si>
+    <t>상장공시, 거래정지/투자유의, IR 자료/일정(보조)</t>
+  </si>
+  <si>
+    <t>웹 구조 변경 리스크 → 파서 버전관리/헬스체크 필요.</t>
+  </si>
+  <si>
+    <t>https://kind.krx.co.kr/</t>
+  </si>
+  <si>
+    <t>미국 공시/재무(XBRL) 원천</t>
+  </si>
+  <si>
+    <t>SEC EDGAR APIs</t>
+  </si>
+  <si>
+    <t>OpenAPI/Web</t>
+  </si>
+  <si>
+    <t>5~15분(신규 filing 감지) + 온디맨드 문서</t>
+  </si>
+  <si>
+    <t>10-K/10-Q/8-K 등 filing, submissions, XBRL facts</t>
+  </si>
+  <si>
+    <t>접속 예절(User-Agent 등) 준수. ticker↔CIK 매핑 필요.</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/search-filings/edgar-application-programming-interfaces</t>
+  </si>
+  <si>
+    <t>공식발표/기관공지</t>
+  </si>
+  <si>
+    <t>미국 기관 릴리즈 스케줄/공지</t>
+  </si>
+  <si>
+    <t>BLS Release Schedules / BEA Schedule</t>
+  </si>
+  <si>
+    <t>Web/JSON/ICS</t>
+  </si>
+  <si>
+    <t>일 1회 + 변경 감지</t>
+  </si>
+  <si>
+    <t>릴리즈 캘린더(예정/변경)</t>
+  </si>
+  <si>
+    <t>일정 변경(정부 셧다운 등) 가능 → 변경 감지 및 재동기화.</t>
+  </si>
+  <si>
+    <t>https://www.bls.gov/schedule/news_release/</t>
+  </si>
+  <si>
+    <t>기업분석/IR</t>
+  </si>
+  <si>
+    <t>IR 자료/기업분석보고서(공개 범위)</t>
+  </si>
+  <si>
+    <t>KIND IR자료실/기업분석보고서</t>
+  </si>
+  <si>
+    <t>Web (다운로드)</t>
+  </si>
+  <si>
+    <t>일 1~4회 + 신규 업로드 시 즉시</t>
+  </si>
+  <si>
+    <t>IR 발표자료(PDF), IR 일정, 분석 보고서(가능 범위)</t>
+  </si>
+  <si>
+    <t>문서 파싱(PDF) 작업 큐 분리 권장. 저작권/이용범위 확인.</t>
+  </si>
+  <si>
+    <t>사업/분반기 보고서 기반 factual</t>
+  </si>
+  <si>
+    <t>DART 사업/분반기 보고서(원문/정형)</t>
+  </si>
+  <si>
+    <t>Event-driven + Batch</t>
+  </si>
+  <si>
+    <t>신규공시 즉시 + 일 1회 보강</t>
+  </si>
+  <si>
+    <t>사업보고서/분기보고서, 재무/리스크 서술</t>
+  </si>
+  <si>
+    <t>리서치 대체가 아니라 factual 기반. LLM 요약/팩트 추출에 적합.</t>
+  </si>
+  <si>
+    <t>투자분석정보/보고서(유료 가능)</t>
+  </si>
+  <si>
+    <t>KRX Data Marketplace (투자분석정보/기업분석보고서)</t>
+  </si>
+  <si>
+    <t>Exchange (Official/Commercial)</t>
+  </si>
+  <si>
+    <t>Data service</t>
+  </si>
+  <si>
+    <t>일 1회 또는 문서 게시 시점</t>
+  </si>
+  <si>
+    <t>분석/리포트류(서비스 범위에 따라)</t>
+  </si>
+  <si>
+    <t>유료/라이선스 조건 확인 후 도입. 재배포/저장 조건 검토 필수.</t>
+  </si>
+  <si>
+    <t>https://data.krx.co.kr/contents/MDC/COMS/client/MDCCOMS002_S3.cmd</t>
+  </si>
+  <si>
+    <t>미국 기업 IR 사이트(보도자료/프리젠테이션)</t>
+  </si>
+  <si>
+    <t>각 기업 Investor Relations(회사별)</t>
+  </si>
+  <si>
+    <t>Company (Official)</t>
+  </si>
+  <si>
+    <t>Web/RSS(있다면)</t>
+  </si>
+  <si>
+    <t>일 1~4회 또는 온디맨드</t>
+  </si>
+  <si>
+    <t>Earnings release, Presentation PDF, prepared remarks, webcast links</t>
+  </si>
+  <si>
+    <t>회사별 구조 상이 → IR URL registry 필요. 약관/robots 준수.</t>
+  </si>
+  <si>
+    <t>(company-specific)</t>
+  </si>
+  <si>
+    <t>식별자/매핑</t>
+  </si>
+  <si>
+    <t>미국 티커↔CIK/filings 참조</t>
+  </si>
+  <si>
+    <t>SEC EDGAR (CIK 중심)</t>
+  </si>
+  <si>
+    <t>주 1회 + 변경 감지</t>
+  </si>
+  <si>
+    <t>CIK, 제출내역, company facts</t>
+  </si>
+  <si>
+    <t>티커 변경/합병 대응 위해 CIK 중심 식별 권장.</t>
+  </si>
+  <si>
+    <t>텔레그램</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TELEGRAM_BOT_TOKEN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TELEGRAM_CHAT_ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8574535049:AAEYELxv66WCdcw-DFE8uEOtMhTL5DJYiHE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>한투</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KIS_APP_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KIS_APP_SECRET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PSG3myj7u7NNZLLouJc7UgNQ9sPQJELFwGfR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VxhY6H+c4dlTgJpJNCGNf6UZsSe05oL35trdmv7eCyR5jhE1zCq6mB39qmgh6tgy8hi5XnDW3NCLkmL0NE31EqwJC5TKL+lvuI/OAouMM5QoQ2mrsubupCXt/AIYnEKHgs0RfqX2oakdT8TqKe0ZrISmbBn2oxjbjr/rTqC5NEw5Z+827FI=</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DART_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fac4ab717e946d173f73227186301dc52678beef</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LSBv0_7RIrFyQAf1MWec</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>vDEvRwBmcl</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAVER_CLIENT_SECRET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAVER_CLIENT_ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X_BEARER_TOKEN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AAAAAAAAAAAAAAAAAAAAACca7wEAAAAA2RHEQ5J%2BIwSS%2BhUtI4Q5jYvcMpY%3DPAnZ4St2dX1NiUl3aEV8Jdy4Pq8PlmERCUqIzwS84jSUztHSrt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://apiportal.koreainvestment.com/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://opendart.fss.or.kr/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DART</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://developers.naver.com/main/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>네이버</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://developer.x.com/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>@BotFather</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>한국은행 Open API</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://ecos.bok.or.kr/api/#/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B9K54QTAQJTPIVPWCPWA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yjg0M2FlZTI4ZTk5NzY3Njk1YTA2MTI0NmYyY2YyMWQ=</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kosis.kr/openapi/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KOSIS(국가통계포털) Open API</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>786f6fe06cae40019f2da976f1a3b1d1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://newsapi.org/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NewsAPI (글로벌 뉴스)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GDELT (글로벌 이벤트/매크로)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://blog.gdeltproject.org/gdelt-2-0-our-global-world-in-realtime/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Programmable Search Engine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://programmablesearchengine.google.com/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>c2c0d0c1358aa4bb5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>BLS Public Data API</t>
-  </si>
-  <si>
-    <t>Batch + Event</t>
-  </si>
-  <si>
-    <t>일 1회 + 발표일 전후 집중</t>
-  </si>
-  <si>
-    <t>CPI/PPI 등 시계열(Series 기반)</t>
-  </si>
-  <si>
-    <t>원천기관 API. 발표값/일정은 별도 릴리즈 페이지/스케줄과 결합 권장.</t>
-  </si>
-  <si>
-    <t>https://www.bls.gov/developers/</t>
-  </si>
-  <si>
-    <t>미국 CPI 릴리즈 페이지/문서</t>
-  </si>
-  <si>
-    <t>BLS CPI News Release</t>
-  </si>
-  <si>
-    <t>Web</t>
-  </si>
-  <si>
-    <t>발표 전후 30초~2분 폴링</t>
-  </si>
-  <si>
-    <t>릴리즈 본문/표/첨부</t>
-  </si>
-  <si>
-    <t>정책/문구 변화 요약에 LLM 사용 가능. 일정 변경 공지 확인 필요.</t>
-  </si>
-  <si>
-    <t>https://www.bls.gov/news.release/cpi.htm</t>
-  </si>
-  <si>
-    <t>미국 GDP/PCE 등</t>
-  </si>
-  <si>
-    <t>BEA API / Release Schedule</t>
-  </si>
-  <si>
-    <t>OpenAPI + Web/JSON/ICS</t>
-  </si>
-  <si>
-    <t>일 1회 + 발표 전후 집중</t>
-  </si>
-  <si>
-    <t>GDP, PCE 등 지표값 및 릴리즈 일정</t>
-  </si>
-  <si>
-    <t>스케줄 JSON/ICS 활용 가능. 개정치(revisions) 처리 고려.</t>
-  </si>
-  <si>
-    <t>https://www.bea.gov/resources/for-developers</t>
-  </si>
-  <si>
-    <t>경제 데이터 통합 허브(백테스트/리비전)</t>
-  </si>
-  <si>
-    <t>FRED API (ALFRED 포함)</t>
-  </si>
-  <si>
-    <t>Federal Reserve (Official)</t>
-  </si>
-  <si>
-    <t>다양한 경제지표 시계열, vintage(리비전) 데이터(옵션)</t>
-  </si>
-  <si>
-    <t>원천기관 대비 중계 레이어. 실시간 발표 해석은 원천기관 우선 권장.</t>
-  </si>
-  <si>
-    <t>https://fred.stlouisfed.org/docs/api/fred/</t>
-  </si>
-  <si>
-    <t>공시</t>
-  </si>
-  <si>
-    <t>한국 공시 원천/원문/XML</t>
-  </si>
-  <si>
-    <t>OPENDART (금감원)</t>
-  </si>
-  <si>
-    <t>Regulator (Official)</t>
-  </si>
-  <si>
-    <t>Polling + On-demand</t>
-  </si>
-  <si>
-    <t>장중/장후 1~3분 폴링 + 원문 즉시 다운로드</t>
-  </si>
-  <si>
-    <t>공시목록, 공시원문(XML/첨부), 정정공시</t>
-  </si>
-  <si>
-    <t>corp_code 매핑 필요. 정정공시 체인 관리 필수.</t>
-  </si>
-  <si>
-    <t>https://opendart.fss.or.kr/</t>
-  </si>
-  <si>
-    <t>거래소 고유공시/투자유의/IR 보완</t>
-  </si>
-  <si>
-    <t>Primary(보완)</t>
-  </si>
-  <si>
-    <t>KRX KIND</t>
-  </si>
-  <si>
-    <t>Web (파싱)</t>
-  </si>
-  <si>
-    <t>2~5분(공시), 1~3분(투자유의)</t>
-  </si>
-  <si>
-    <t>상장공시, 거래정지/투자유의, IR 자료/일정(보조)</t>
-  </si>
-  <si>
-    <t>웹 구조 변경 리스크 → 파서 버전관리/헬스체크 필요.</t>
-  </si>
-  <si>
-    <t>https://kind.krx.co.kr/</t>
-  </si>
-  <si>
-    <t>미국 공시/재무(XBRL) 원천</t>
-  </si>
-  <si>
-    <t>SEC EDGAR APIs</t>
-  </si>
-  <si>
-    <t>OpenAPI/Web</t>
-  </si>
-  <si>
-    <t>5~15분(신규 filing 감지) + 온디맨드 문서</t>
-  </si>
-  <si>
-    <t>10-K/10-Q/8-K 등 filing, submissions, XBRL facts</t>
-  </si>
-  <si>
-    <t>접속 예절(User-Agent 등) 준수. ticker↔CIK 매핑 필요.</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/search-filings/edgar-application-programming-interfaces</t>
-  </si>
-  <si>
-    <t>공식발표/기관공지</t>
-  </si>
-  <si>
-    <t>미국 기관 릴리즈 스케줄/공지</t>
-  </si>
-  <si>
-    <t>BLS Release Schedules / BEA Schedule</t>
-  </si>
-  <si>
-    <t>Web/JSON/ICS</t>
-  </si>
-  <si>
-    <t>일 1회 + 변경 감지</t>
-  </si>
-  <si>
-    <t>릴리즈 캘린더(예정/변경)</t>
-  </si>
-  <si>
-    <t>일정 변경(정부 셧다운 등) 가능 → 변경 감지 및 재동기화.</t>
-  </si>
-  <si>
-    <t>https://www.bls.gov/schedule/news_release/</t>
-  </si>
-  <si>
-    <t>기업분석/IR</t>
-  </si>
-  <si>
-    <t>IR 자료/기업분석보고서(공개 범위)</t>
-  </si>
-  <si>
-    <t>KIND IR자료실/기업분석보고서</t>
-  </si>
-  <si>
-    <t>Web (다운로드)</t>
-  </si>
-  <si>
-    <t>일 1~4회 + 신규 업로드 시 즉시</t>
-  </si>
-  <si>
-    <t>IR 발표자료(PDF), IR 일정, 분석 보고서(가능 범위)</t>
-  </si>
-  <si>
-    <t>문서 파싱(PDF) 작업 큐 분리 권장. 저작권/이용범위 확인.</t>
-  </si>
-  <si>
-    <t>사업/분반기 보고서 기반 factual</t>
-  </si>
-  <si>
-    <t>DART 사업/분반기 보고서(원문/정형)</t>
-  </si>
-  <si>
-    <t>Event-driven + Batch</t>
-  </si>
-  <si>
-    <t>신규공시 즉시 + 일 1회 보강</t>
-  </si>
-  <si>
-    <t>사업보고서/분기보고서, 재무/리스크 서술</t>
-  </si>
-  <si>
-    <t>리서치 대체가 아니라 factual 기반. LLM 요약/팩트 추출에 적합.</t>
-  </si>
-  <si>
-    <t>투자분석정보/보고서(유료 가능)</t>
-  </si>
-  <si>
-    <t>KRX Data Marketplace (투자분석정보/기업분석보고서)</t>
-  </si>
-  <si>
-    <t>Exchange (Official/Commercial)</t>
-  </si>
-  <si>
-    <t>Data service</t>
-  </si>
-  <si>
-    <t>일 1회 또는 문서 게시 시점</t>
-  </si>
-  <si>
-    <t>분석/리포트류(서비스 범위에 따라)</t>
-  </si>
-  <si>
-    <t>유료/라이선스 조건 확인 후 도입. 재배포/저장 조건 검토 필수.</t>
-  </si>
-  <si>
-    <t>https://data.krx.co.kr/contents/MDC/COMS/client/MDCCOMS002_S3.cmd</t>
-  </si>
-  <si>
-    <t>미국 기업 IR 사이트(보도자료/프리젠테이션)</t>
-  </si>
-  <si>
-    <t>각 기업 Investor Relations(회사별)</t>
-  </si>
-  <si>
-    <t>Company (Official)</t>
-  </si>
-  <si>
-    <t>Web/RSS(있다면)</t>
-  </si>
-  <si>
-    <t>일 1~4회 또는 온디맨드</t>
-  </si>
-  <si>
-    <t>Earnings release, Presentation PDF, prepared remarks, webcast links</t>
-  </si>
-  <si>
-    <t>회사별 구조 상이 → IR URL registry 필요. 약관/robots 준수.</t>
-  </si>
-  <si>
-    <t>(company-specific)</t>
-  </si>
-  <si>
-    <t>식별자/매핑</t>
-  </si>
-  <si>
-    <t>미국 티커↔CIK/filings 참조</t>
-  </si>
-  <si>
-    <t>SEC EDGAR (CIK 중심)</t>
-  </si>
-  <si>
-    <t>주 1회 + 변경 감지</t>
-  </si>
-  <si>
-    <t>CIK, 제출내역, company facts</t>
-  </si>
-  <si>
-    <t>티커 변경/합병 대응 위해 CIK 중심 식별 권장.</t>
-  </si>
-  <si>
-    <t>텔레그램</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TELEGRAM_BOT_TOKEN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TELEGRAM_CHAT_ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>8574535049:AAEYELxv66WCdcw-DFE8uEOtMhTL5DJYiHE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>한투</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>KIS_APP_KEY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>KIS_APP_SECRET</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PSG3myj7u7NNZLLouJc7UgNQ9sPQJELFwGfR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VxhY6H+c4dlTgJpJNCGNf6UZsSe05oL35trdmv7eCyR5jhE1zCq6mB39qmgh6tgy8hi5XnDW3NCLkmL0NE31EqwJC5TKL+lvuI/OAouMM5QoQ2mrsubupCXt/AIYnEKHgs0RfqX2oakdT8TqKe0ZrISmbBn2oxjbjr/rTqC5NEw5Z+827FI=</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DART_API_KEY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fac4ab717e946d173f73227186301dc52678beef</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>LSBv0_7RIrFyQAf1MWec</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>vDEvRwBmcl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NAVER_CLIENT_SECRET</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NAVER_CLIENT_ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X_BEARER_TOKEN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AAAAAAAAAAAAAAAAAAAAACca7wEAAAAA2RHEQ5J%2BIwSS%2BhUtI4Q5jYvcMpY%3DPAnZ4St2dX1NiUl3aEV8Jdy4Pq8PlmERCUqIzwS84jSUztHSrt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://apiportal.koreainvestment.com/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://opendart.fss.or.kr/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DART</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://developers.naver.com/main/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>네이버</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://developer.x.com/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>@BotFather</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>한국은행 Open API</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://ecos.bok.or.kr/api/#/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>B9K54QTAQJTPIVPWCPWA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Yjg0M2FlZTI4ZTk5NzY3Njk1YTA2MTI0NmYyY2YyMWQ=</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://kosis.kr/openapi/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>KOSIS(국가통계포털) Open API</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>786f6fe06cae40019f2da976f1a3b1d1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://newsapi.org/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NewsAPI (글로벌 뉴스)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>GDELT (글로벌 이벤트/매크로)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://blog.gdeltproject.org/gdelt-2-0-our-global-world-in-realtime/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Programmable Search Engine</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://programmablesearchengine.google.com/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>c2c0d0c1358aa4bb5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1542,8 +1543,8 @@
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="13.125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="51.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.125" bestFit="1" customWidth="1"/>
@@ -2214,7 +2215,7 @@
         <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>171</v>
+        <v>302</v>
       </c>
       <c r="F18" t="s">
         <v>157</v>
@@ -2223,19 +2224,19 @@
         <v>71</v>
       </c>
       <c r="H18" t="s">
+        <v>171</v>
+      </c>
+      <c r="I18" t="s">
         <v>172</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>173</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>174</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>175</v>
-      </c>
-      <c r="L18" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
@@ -2243,7 +2244,7 @@
         <v>140</v>
       </c>
       <c r="B19" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C19" t="s">
         <v>77</v>
@@ -2252,28 +2253,28 @@
         <v>39</v>
       </c>
       <c r="E19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F19" t="s">
         <v>157</v>
       </c>
       <c r="G19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H19" t="s">
         <v>159</v>
       </c>
       <c r="I19" t="s">
+        <v>179</v>
+      </c>
+      <c r="J19" t="s">
         <v>180</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>181</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>182</v>
-      </c>
-      <c r="L19" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
@@ -2281,7 +2282,7 @@
         <v>140</v>
       </c>
       <c r="B20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C20" t="s">
         <v>77</v>
@@ -2290,28 +2291,28 @@
         <v>39</v>
       </c>
       <c r="E20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F20" t="s">
         <v>157</v>
       </c>
       <c r="G20" t="s">
+        <v>185</v>
+      </c>
+      <c r="H20" t="s">
+        <v>171</v>
+      </c>
+      <c r="I20" t="s">
         <v>186</v>
       </c>
-      <c r="H20" t="s">
-        <v>172</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>187</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>188</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>189</v>
-      </c>
-      <c r="L20" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
@@ -2319,7 +2320,7 @@
         <v>140</v>
       </c>
       <c r="B21" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C21" t="s">
         <v>77</v>
@@ -2328,10 +2329,10 @@
         <v>49</v>
       </c>
       <c r="E21" t="s">
+        <v>191</v>
+      </c>
+      <c r="F21" t="s">
         <v>192</v>
-      </c>
-      <c r="F21" t="s">
-        <v>193</v>
       </c>
       <c r="G21" t="s">
         <v>71</v>
@@ -2343,21 +2344,21 @@
         <v>151</v>
       </c>
       <c r="J21" t="s">
+        <v>193</v>
+      </c>
+      <c r="K21" t="s">
         <v>194</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>195</v>
-      </c>
-      <c r="L21" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" t="s">
         <v>197</v>
-      </c>
-      <c r="B22" t="s">
-        <v>198</v>
       </c>
       <c r="C22" t="s">
         <v>38</v>
@@ -2366,74 +2367,74 @@
         <v>39</v>
       </c>
       <c r="E22" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F22" t="s">
         <v>199</v>
-      </c>
-      <c r="F22" t="s">
-        <v>200</v>
       </c>
       <c r="G22" t="s">
         <v>71</v>
       </c>
       <c r="H22" t="s">
+        <v>200</v>
+      </c>
+      <c r="I22" t="s">
         <v>201</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>202</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>203</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>204</v>
-      </c>
-      <c r="L22" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B23" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C23" t="s">
         <v>38</v>
       </c>
       <c r="D23" t="s">
+        <v>206</v>
+      </c>
+      <c r="E23" t="s">
         <v>207</v>
-      </c>
-      <c r="E23" t="s">
-        <v>208</v>
       </c>
       <c r="F23" t="s">
         <v>59</v>
       </c>
       <c r="G23" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H23" t="s">
         <v>89</v>
       </c>
       <c r="I23" t="s">
+        <v>209</v>
+      </c>
+      <c r="J23" t="s">
         <v>210</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>211</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>212</v>
-      </c>
-      <c r="L23" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C24" t="s">
         <v>77</v>
@@ -2442,36 +2443,36 @@
         <v>39</v>
       </c>
       <c r="E24" t="s">
+        <v>214</v>
+      </c>
+      <c r="F24" t="s">
+        <v>199</v>
+      </c>
+      <c r="G24" t="s">
         <v>215</v>
       </c>
-      <c r="F24" t="s">
+      <c r="H24" t="s">
         <v>200</v>
       </c>
-      <c r="G24" t="s">
+      <c r="I24" t="s">
         <v>216</v>
       </c>
-      <c r="H24" t="s">
-        <v>201</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>217</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>218</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>219</v>
-      </c>
-      <c r="L24" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" t="s">
         <v>221</v>
-      </c>
-      <c r="B25" t="s">
-        <v>222</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -2480,36 +2481,36 @@
         <v>39</v>
       </c>
       <c r="E25" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F25" t="s">
         <v>157</v>
       </c>
       <c r="G25" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" t="s">
+        <v>171</v>
+      </c>
+      <c r="I25" t="s">
         <v>224</v>
       </c>
-      <c r="H25" t="s">
-        <v>172</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>225</v>
       </c>
-      <c r="J25" t="s">
+      <c r="K25" t="s">
         <v>226</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>227</v>
-      </c>
-      <c r="L25" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>228</v>
+      </c>
+      <c r="B26" t="s">
         <v>229</v>
-      </c>
-      <c r="B26" t="s">
-        <v>230</v>
       </c>
       <c r="C26" t="s">
         <v>38</v>
@@ -2518,36 +2519,36 @@
         <v>39</v>
       </c>
       <c r="E26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F26" t="s">
         <v>59</v>
       </c>
       <c r="G26" t="s">
+        <v>231</v>
+      </c>
+      <c r="H26" t="s">
+        <v>171</v>
+      </c>
+      <c r="I26" t="s">
         <v>232</v>
       </c>
-      <c r="H26" t="s">
-        <v>172</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>233</v>
       </c>
-      <c r="J26" t="s">
+      <c r="K26" t="s">
         <v>234</v>
       </c>
-      <c r="K26" t="s">
-        <v>235</v>
-      </c>
       <c r="L26" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B27" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C27" t="s">
         <v>38</v>
@@ -2556,36 +2557,36 @@
         <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F27" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G27" t="s">
         <v>71</v>
       </c>
       <c r="H27" t="s">
+        <v>237</v>
+      </c>
+      <c r="I27" t="s">
         <v>238</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>239</v>
       </c>
-      <c r="J27" t="s">
+      <c r="K27" t="s">
         <v>240</v>
       </c>
-      <c r="K27" t="s">
-        <v>241</v>
-      </c>
       <c r="L27" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B28" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C28" t="s">
         <v>38</v>
@@ -2594,36 +2595,36 @@
         <v>49</v>
       </c>
       <c r="E28" t="s">
+        <v>242</v>
+      </c>
+      <c r="F28" t="s">
         <v>243</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>244</v>
-      </c>
-      <c r="G28" t="s">
-        <v>245</v>
       </c>
       <c r="H28" t="s">
         <v>61</v>
       </c>
       <c r="I28" t="s">
+        <v>245</v>
+      </c>
+      <c r="J28" t="s">
         <v>246</v>
       </c>
-      <c r="J28" t="s">
+      <c r="K28" t="s">
         <v>247</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>248</v>
-      </c>
-      <c r="L28" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B29" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C29" t="s">
         <v>77</v>
@@ -2632,36 +2633,36 @@
         <v>39</v>
       </c>
       <c r="E29" t="s">
+        <v>250</v>
+      </c>
+      <c r="F29" t="s">
         <v>251</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>252</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
+        <v>171</v>
+      </c>
+      <c r="I29" t="s">
         <v>253</v>
       </c>
-      <c r="H29" t="s">
-        <v>172</v>
-      </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>254</v>
       </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>255</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>256</v>
-      </c>
-      <c r="L29" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>257</v>
+      </c>
+      <c r="B30" t="s">
         <v>258</v>
-      </c>
-      <c r="B30" t="s">
-        <v>259</v>
       </c>
       <c r="C30" t="s">
         <v>77</v>
@@ -2670,28 +2671,28 @@
         <v>39</v>
       </c>
       <c r="E30" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G30" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H30" t="s">
         <v>61</v>
       </c>
       <c r="I30" t="s">
+        <v>260</v>
+      </c>
+      <c r="J30" t="s">
         <v>261</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>262</v>
       </c>
-      <c r="K30" t="s">
-        <v>263</v>
-      </c>
       <c r="L30" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -2713,21 +2714,21 @@
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" t="s">
         <v>264</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D3" t="s">
-        <v>265</v>
-      </c>
       <c r="E3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="D4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E4">
         <v>5728656884</v>
@@ -2735,38 +2736,38 @@
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" t="s">
         <v>268</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="D6" t="s">
-        <v>269</v>
-      </c>
       <c r="E6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D9" t="s">
+        <v>272</v>
+      </c>
+      <c r="E9" t="s">
         <v>273</v>
-      </c>
-      <c r="E9" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
@@ -2774,90 +2775,90 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E14" t="s">
         <v>279</v>
-      </c>
-      <c r="E14" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
+        <v>288</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="E16" t="s">
         <v>290</v>
-      </c>
-      <c r="E16" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E18" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E20" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
+        <v>297</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
+        <v>299</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" t="s">
         <v>301</v>
-      </c>
-      <c r="E24" t="s">
-        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: upgrade decision products and market intelligence
</commit_message>
<xml_diff>
--- a/investai.xlsx
+++ b/investai.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\invest_ai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D999B8F9-9616-46D0-AB78-10B562F64120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3CB7D2F-4D07-48A7-AE45-4B12252FEA3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12600" yWindow="0" windowWidth="12600" windowHeight="15150" activeTab="1" xr2:uid="{F5D4FDE9-00C8-4EAA-8556-5AECFB8EB8A2}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12600" windowHeight="15150" activeTab="2" xr2:uid="{F5D4FDE9-00C8-4EAA-8556-5AECFB8EB8A2}"/>
   </bookViews>
   <sheets>
     <sheet name="개요" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="340">
   <si>
     <t>데이터 원천 소스 설계</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1010,6 +1010,152 @@
   </si>
   <si>
     <t>BLS Public Data API</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://data-explorer.oecd.org/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xkrrmswn8549t747T!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xkrrmswn@gmail.com</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://fredaccount.stlouisfed.org</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>efb9042054669c80e9f52f843cfed3ce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>.env 반영여부</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ㅇ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>a0b0b10bc4be49c590858c1f91907523</t>
+  </si>
+  <si>
+    <t>https://data.bls.gov/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1750107B-3384-4661-B804-E03AE80E201F</t>
+  </si>
+  <si>
+    <t>https://apps.bea.gov/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://fiscaldata.treasury.gov/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FRED_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BLS_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BEA_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NEWS_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KOSIS_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BOK_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OECD_ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OECD_PW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PSE_API_KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>물가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GDP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>재정</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Eurostat API (유럽통계처)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://ec.europa.eu/eurostat/web/user-guides/data-browser/api-data-access/api-getting-started</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OECD API (경제협력개발기구)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FRED (세인트루이스 연방준비은행)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BLS (미국 노동통계국)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BEA (미국 경제분석국)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fiscal Data (미국 재무부)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ECB Data Portal API (유럽중앙은행)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.ecb.europa.eu/stats/accessing-our-data/html/index.en.html</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>World Bank API</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://api.worldbank.org</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> IMF (International Monetary Fund) API</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1017,7 +1163,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1041,6 +1187,19 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1080,7 +1239,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1094,6 +1253,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2703,177 +2871,355 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7360E6EB-3C34-4966-B7EE-4EC5E6785CE1}">
-  <dimension ref="B3:E24"/>
+  <dimension ref="A2:F43"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="210.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.375" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="4" max="4" width="33.375" customWidth="1"/>
+    <col min="5" max="5" width="23.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="210.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>309</v>
+      </c>
       <c r="B3" t="s">
         <v>263</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>264</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
         <v>265</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>5728656884</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>309</v>
+      </c>
       <c r="B6" t="s">
         <v>267</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>268</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D7" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
         <v>269</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>309</v>
+      </c>
       <c r="B9" t="s">
         <v>283</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>272</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>309</v>
+      </c>
       <c r="B11" t="s">
         <v>285</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>277</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D12" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
         <v>276</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>309</v>
+      </c>
       <c r="B14" t="s">
         <v>280</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>278</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>309</v>
+      </c>
       <c r="B16" t="s">
         <v>288</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>289</v>
       </c>
       <c r="E16" t="s">
+        <v>320</v>
+      </c>
+      <c r="F16" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>309</v>
+      </c>
       <c r="B18" t="s">
         <v>293</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>292</v>
       </c>
       <c r="E18" t="s">
+        <v>319</v>
+      </c>
+      <c r="F18" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>309</v>
+      </c>
       <c r="B20" t="s">
         <v>296</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>295</v>
       </c>
       <c r="E20" t="s">
+        <v>318</v>
+      </c>
+      <c r="F20" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>297</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>299</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>300</v>
       </c>
       <c r="E24" t="s">
+        <v>323</v>
+      </c>
+      <c r="F24" t="s">
         <v>301</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>330</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E26" t="s">
+        <v>321</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E27" t="s">
+        <v>322</v>
+      </c>
+      <c r="F27" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>331</v>
+      </c>
+      <c r="C29" t="s">
+        <v>324</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E29" t="s">
+        <v>315</v>
+      </c>
+      <c r="F29" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>332</v>
+      </c>
+      <c r="C31" t="s">
+        <v>325</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E31" t="s">
+        <v>316</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>333</v>
+      </c>
+      <c r="C33" t="s">
+        <v>326</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E33" t="s">
+        <v>317</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>334</v>
+      </c>
+      <c r="C35" t="s">
+        <v>327</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E35" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>335</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="E37" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>328</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E39" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>337</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E41" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>339</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C6" r:id="rId1" xr:uid="{C6C82609-9060-4FC9-ADC3-E221DE1BAD26}"/>
-    <hyperlink ref="C9" r:id="rId2" xr:uid="{517EB071-0C9C-4342-9668-E0F471041E20}"/>
-    <hyperlink ref="C11" r:id="rId3" xr:uid="{4E878D1C-F8C5-4905-98B3-B86210CAE961}"/>
-    <hyperlink ref="C14" r:id="rId4" xr:uid="{D49B3597-CC61-4365-9E4F-2DA7AF6F85B8}"/>
-    <hyperlink ref="C16" r:id="rId5" location="/" xr:uid="{5FC3C801-A841-439F-9505-6CA23228FD23}"/>
-    <hyperlink ref="C18" r:id="rId6" xr:uid="{E824DD37-4504-4C07-9A7E-E7085BA26180}"/>
-    <hyperlink ref="C20" r:id="rId7" xr:uid="{93FB7923-08EF-4FF8-B6E4-5FC4CC950140}"/>
-    <hyperlink ref="C22" r:id="rId8" xr:uid="{3432FE00-EE4F-4AA2-946F-CDFD2584CA8C}"/>
-    <hyperlink ref="C24" r:id="rId9" xr:uid="{C7AFB880-633B-4E3A-AD53-FB7A59A60873}"/>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{C6C82609-9060-4FC9-ADC3-E221DE1BAD26}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{517EB071-0C9C-4342-9668-E0F471041E20}"/>
+    <hyperlink ref="D11" r:id="rId3" xr:uid="{4E878D1C-F8C5-4905-98B3-B86210CAE961}"/>
+    <hyperlink ref="D14" r:id="rId4" xr:uid="{D49B3597-CC61-4365-9E4F-2DA7AF6F85B8}"/>
+    <hyperlink ref="D16" r:id="rId5" location="/" xr:uid="{5FC3C801-A841-439F-9505-6CA23228FD23}"/>
+    <hyperlink ref="D18" r:id="rId6" xr:uid="{E824DD37-4504-4C07-9A7E-E7085BA26180}"/>
+    <hyperlink ref="D20" r:id="rId7" xr:uid="{93FB7923-08EF-4FF8-B6E4-5FC4CC950140}"/>
+    <hyperlink ref="D22" r:id="rId8" xr:uid="{3432FE00-EE4F-4AA2-946F-CDFD2584CA8C}"/>
+    <hyperlink ref="D24" r:id="rId9" xr:uid="{C7AFB880-633B-4E3A-AD53-FB7A59A60873}"/>
+    <hyperlink ref="D26" r:id="rId10" xr:uid="{624DF0F3-8552-4652-B574-777A9ADB2935}"/>
+    <hyperlink ref="F26" r:id="rId11" xr:uid="{B04BDB79-CE42-4B47-9FA5-37B84B4E35A5}"/>
+    <hyperlink ref="D29" r:id="rId12" xr:uid="{827EAB26-6E9C-494C-9D3D-77BB4E853382}"/>
+    <hyperlink ref="D31" r:id="rId13" xr:uid="{C26A11D7-3047-4045-9016-324EA75F0B75}"/>
+    <hyperlink ref="D33" r:id="rId14" xr:uid="{AAF50F7C-762E-4C3D-B23B-7611E049017A}"/>
+    <hyperlink ref="D35" r:id="rId15" xr:uid="{7AD52247-19EE-4457-8732-72B04CFF13B3}"/>
+    <hyperlink ref="D39" r:id="rId16" xr:uid="{730AD477-E328-4DFC-8F27-ECCA94194AC7}"/>
+    <hyperlink ref="D37" r:id="rId17" xr:uid="{ABF1FABD-B72D-4E87-8163-80E637638251}"/>
+    <hyperlink ref="D41" r:id="rId18" xr:uid="{FCB1988E-63C6-41D4-922B-83336CF4BAFF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>